<commit_message>
- Introduce Composition Root in bootstrap.py and use-case dispatcher.- Decouple business logic from Selenium/scrapers using Ports and Adapters.- Standardize use-case contracts with a unified execute() method.- Add DTOs (QuotationRequest) with built-in validation and custom errors.- Modernize configuration handling with a dedicated .env loader.- Remove legacy brand modules and redundant shims.- Increase test coverage with unit and integration tests.
</commit_message>
<xml_diff>
--- a/for_client/HORSCH_204.xlsx_quotation.xlsx
+++ b/for_client/HORSCH_204.xlsx_quotation.xlsx
@@ -413,341 +413,293 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>codes</t>
+        </is>
+      </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>codes</t>
+          <t>qty</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>qty</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
           <t>prices</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>0</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>00240231</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>00240231</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>117,09</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>95110360</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>117,09</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>95110360</t>
-        </is>
-      </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>137,28</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>00240177</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>137,28</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>00240177</t>
-        </is>
-      </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
           <t>96,09</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>3</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>00310131</t>
+        </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>00310131</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>12,92</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>00311208</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Brak ceny</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>23010202</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>12,92</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>00311208</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>7,01</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>23010204</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0,92</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>23010205</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0,99</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>23246102</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>36,34</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>23010203</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>0,21</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>00360363</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>0,09</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>23010201</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>21,80</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>23044002</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>12,26</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>23044200</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>15,14</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>00360111</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Brak ceny</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>23010202</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>7,01</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>23010204</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>0,92</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>23010205</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>0,99</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>23246102</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>48</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>36,34</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>23010203</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>96</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>0,21</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>10</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>00360363</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>184</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>0,09</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>11</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>23010201</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>96</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>21,80</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>12</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>23044002</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>12,26</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>23044200</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>48</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>15,14</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>14</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>00360111</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>00370104</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>0,09</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>15</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>00370104</t>
-        </is>
-      </c>
       <c r="C17" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
         <is>
           <t>0,01</t>
         </is>

</xml_diff>